<commit_message>
feat: init project with db scripts and documents
</commit_message>
<xml_diff>
--- a/欄位.xlsx
+++ b/欄位.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0C2131F-EDD5-4814-881B-D90C459494DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF1AFE99-BC76-46B4-9E91-A9F8880819E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-109" yWindow="-109" windowWidth="26301" windowHeight="14169" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="HCM 月子平台 -市府" sheetId="1" r:id="rId1"/>
-    <sheet name="beclass" sheetId="2" r:id="rId2"/>
+    <sheet name="服務人員" sheetId="3" r:id="rId2"/>
+    <sheet name="beclass" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="176">
   <si>
     <r>
       <rPr>
@@ -673,13 +674,150 @@
   </si>
   <si>
     <t>HC115011</t>
+  </si>
+  <si>
+    <t>IP位址</t>
+  </si>
+  <si>
+    <t>銀行帳號</t>
+  </si>
+  <si>
+    <t>銀行代3碼+分行代號4碼</t>
+  </si>
+  <si>
+    <t>身分證字號</t>
+  </si>
+  <si>
+    <t>EMAIL</t>
+  </si>
+  <si>
+    <t>若有其它同銀行帳號，請一併提供。(永豐或台新)</t>
+  </si>
+  <si>
+    <t>承上題</t>
+  </si>
+  <si>
+    <t>月子餐點料理</t>
+  </si>
+  <si>
+    <t>可承接案件區域</t>
+  </si>
+  <si>
+    <t>北區</t>
+  </si>
+  <si>
+    <t>東區</t>
+  </si>
+  <si>
+    <t>香山區</t>
+  </si>
+  <si>
+    <t>新竹縣</t>
+  </si>
+  <si>
+    <t>苗栗縣</t>
+  </si>
+  <si>
+    <t>可承接案件時段</t>
+  </si>
+  <si>
+    <t>4小時(上午8:30-12:30)</t>
+  </si>
+  <si>
+    <t>4小時(下午13:00-17:00)</t>
+  </si>
+  <si>
+    <t>8小時</t>
+  </si>
+  <si>
+    <t>24小時</t>
+  </si>
+  <si>
+    <t>可服務週間</t>
+  </si>
+  <si>
+    <t>連續服務</t>
+  </si>
+  <si>
+    <t>週休1日</t>
+  </si>
+  <si>
+    <t>週休2日</t>
+  </si>
+  <si>
+    <t>可承接的胎數</t>
+  </si>
+  <si>
+    <t>單胞胎</t>
+  </si>
+  <si>
+    <t>雙胞胎</t>
+  </si>
+  <si>
+    <t>服務時交通工具</t>
+  </si>
+  <si>
+    <t>機車</t>
+  </si>
+  <si>
+    <t>轎車</t>
+  </si>
+  <si>
+    <t>特殊節日可上班的部分(計費:服務費雙倍)</t>
+  </si>
+  <si>
+    <t>國定假日必休</t>
+  </si>
+  <si>
+    <t>有嬰幼兒按摩證書嗎?</t>
+  </si>
+  <si>
+    <t>民國出生年月日</t>
+    <phoneticPr fontId="12" type="noConversion"/>
+  </si>
+  <si>
+    <t>我提供的帳號是永豐銀行帳戶</t>
+  </si>
+  <si>
+    <t>葷食、素食</t>
+  </si>
+  <si>
+    <t>北區、東區、香山區、新竹縣</t>
+  </si>
+  <si>
+    <t>4小時(上午8:30-12:30)、4小時(下午13:00-17:00)、8小時</t>
+  </si>
+  <si>
+    <t>連續服務、週休1日、週休2日</t>
+  </si>
+  <si>
+    <t>單胞胎、雙胞胎</t>
+  </si>
+  <si>
+    <t>機車、轎車</t>
+  </si>
+  <si>
+    <t>年節農曆過年初一、年節農曆過年初二、年節農曆過年初三、端午節、中秋節</t>
+  </si>
+  <si>
+    <t>E013謝英英</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>E013</t>
+  </si>
+  <si>
+    <t>謝英英</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="11" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="177" formatCode="[$-404]e/m/d;@"/>
+  </numFmts>
+  <fonts count="13">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -748,10 +886,23 @@
       <charset val="136"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Microsoft JhengHei"/>
+      <family val="2"/>
+      <charset val="136"/>
+    </font>
+    <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="微軟正黑體"/>
       <family val="2"/>
+      <charset val="136"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="細明體"/>
+      <family val="3"/>
       <charset val="136"/>
     </font>
   </fonts>
@@ -816,7 +967,7 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -843,11 +994,24 @@
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="2"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="一般" xfId="0" builtinId="0"/>
@@ -1131,7 +1295,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:X2"/>
-  <sheetFormatPr defaultRowHeight="14.95" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.95"/>
   <cols>
     <col min="3" max="3" width="14.5" customWidth="1"/>
     <col min="6" max="6" width="16" customWidth="1"/>
@@ -1139,7 +1303,7 @@
     <col min="23" max="23" width="12.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" s="1" customFormat="1" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:24" s="1" customFormat="1" ht="16.149999999999999" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1213,7 +1377,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:24" s="1" customFormat="1" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:24" s="1" customFormat="1" ht="16.149999999999999" customHeight="1">
       <c r="A2" s="1">
         <f t="shared" ref="A2" si="0">ROW(A2)-1</f>
         <v>1</v>
@@ -1291,15 +1455,345 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F0B50C6-6D09-460C-97EF-B843F3DC480C}">
+  <dimension ref="A1:BG2"/>
+  <sheetFormatPr defaultRowHeight="14.95"/>
+  <cols>
+    <col min="4" max="4" width="22.5" customWidth="1"/>
+    <col min="19" max="19" width="17" customWidth="1"/>
+    <col min="20" max="20" width="19.75" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:59" ht="89.7">
+      <c r="A1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C1" t="s">
+        <v>25</v>
+      </c>
+      <c r="D1" t="s">
+        <v>132</v>
+      </c>
+      <c r="E1" t="s">
+        <v>26</v>
+      </c>
+      <c r="F1" s="15" t="s">
+        <v>133</v>
+      </c>
+      <c r="G1" s="16" t="s">
+        <v>134</v>
+      </c>
+      <c r="H1" t="s">
+        <v>135</v>
+      </c>
+      <c r="I1" t="s">
+        <v>32</v>
+      </c>
+      <c r="J1" t="s">
+        <v>136</v>
+      </c>
+      <c r="K1" t="s">
+        <v>29</v>
+      </c>
+      <c r="L1" t="s">
+        <v>30</v>
+      </c>
+      <c r="M1" t="s">
+        <v>31</v>
+      </c>
+      <c r="N1" t="s">
+        <v>33</v>
+      </c>
+      <c r="O1" t="s">
+        <v>34</v>
+      </c>
+      <c r="P1" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>36</v>
+      </c>
+      <c r="R1" t="s">
+        <v>37</v>
+      </c>
+      <c r="S1" s="17" t="s">
+        <v>137</v>
+      </c>
+      <c r="T1" t="s">
+        <v>138</v>
+      </c>
+      <c r="U1" t="s">
+        <v>139</v>
+      </c>
+      <c r="V1" t="s">
+        <v>39</v>
+      </c>
+      <c r="W1" t="s">
+        <v>40</v>
+      </c>
+      <c r="X1" t="s">
+        <v>43</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>140</v>
+      </c>
+      <c r="Z1" t="s">
+        <v>141</v>
+      </c>
+      <c r="AA1" t="s">
+        <v>142</v>
+      </c>
+      <c r="AB1" t="s">
+        <v>143</v>
+      </c>
+      <c r="AC1" t="s">
+        <v>144</v>
+      </c>
+      <c r="AD1" t="s">
+        <v>145</v>
+      </c>
+      <c r="AE1" t="s">
+        <v>43</v>
+      </c>
+      <c r="AF1" t="s">
+        <v>146</v>
+      </c>
+      <c r="AG1" t="s">
+        <v>147</v>
+      </c>
+      <c r="AH1" t="s">
+        <v>148</v>
+      </c>
+      <c r="AI1" t="s">
+        <v>149</v>
+      </c>
+      <c r="AJ1" t="s">
+        <v>150</v>
+      </c>
+      <c r="AK1" t="s">
+        <v>43</v>
+      </c>
+      <c r="AL1" t="s">
+        <v>151</v>
+      </c>
+      <c r="AM1" t="s">
+        <v>152</v>
+      </c>
+      <c r="AN1" t="s">
+        <v>153</v>
+      </c>
+      <c r="AO1" t="s">
+        <v>154</v>
+      </c>
+      <c r="AP1" t="s">
+        <v>43</v>
+      </c>
+      <c r="AQ1" t="s">
+        <v>155</v>
+      </c>
+      <c r="AR1" t="s">
+        <v>156</v>
+      </c>
+      <c r="AS1" t="s">
+        <v>157</v>
+      </c>
+      <c r="AT1" t="s">
+        <v>43</v>
+      </c>
+      <c r="AU1" t="s">
+        <v>158</v>
+      </c>
+      <c r="AV1" t="s">
+        <v>159</v>
+      </c>
+      <c r="AW1" t="s">
+        <v>160</v>
+      </c>
+      <c r="AX1" t="s">
+        <v>161</v>
+      </c>
+      <c r="AY1" t="s">
+        <v>83</v>
+      </c>
+      <c r="AZ1" t="s">
+        <v>84</v>
+      </c>
+      <c r="BA1" t="s">
+        <v>85</v>
+      </c>
+      <c r="BB1" t="s">
+        <v>86</v>
+      </c>
+      <c r="BC1" t="s">
+        <v>87</v>
+      </c>
+      <c r="BD1" t="s">
+        <v>162</v>
+      </c>
+      <c r="BE1" t="s">
+        <v>43</v>
+      </c>
+      <c r="BF1" t="s">
+        <v>163</v>
+      </c>
+      <c r="BG1" s="18" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="2" spans="1:59">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>173</v>
+      </c>
+      <c r="C2" t="str">
+        <f t="shared" ref="C2" si="0">IF(ISNUMBER(SEARCH("807",$G2)),
+   "永豐銀行",
+   IF(ISNUMBER(SEARCH("812",$G2)),
+      "台新",
+      ""
+   )
+)</f>
+        <v/>
+      </c>
+      <c r="D2" t="s">
+        <v>174</v>
+      </c>
+      <c r="E2" t="s">
+        <v>175</v>
+      </c>
+      <c r="F2" s="19"/>
+      <c r="G2" s="20"/>
+      <c r="K2">
+        <v>61</v>
+      </c>
+      <c r="L2">
+        <v>12</v>
+      </c>
+      <c r="M2">
+        <v>24</v>
+      </c>
+      <c r="P2" t="s">
+        <v>144</v>
+      </c>
+      <c r="Q2">
+        <v>302</v>
+      </c>
+      <c r="T2" t="s">
+        <v>165</v>
+      </c>
+      <c r="U2" t="s">
+        <v>166</v>
+      </c>
+      <c r="V2" t="s">
+        <v>120</v>
+      </c>
+      <c r="W2" t="s">
+        <v>120</v>
+      </c>
+      <c r="Y2" t="s">
+        <v>167</v>
+      </c>
+      <c r="Z2" t="s">
+        <v>120</v>
+      </c>
+      <c r="AA2" t="s">
+        <v>120</v>
+      </c>
+      <c r="AB2" t="s">
+        <v>120</v>
+      </c>
+      <c r="AC2" t="s">
+        <v>120</v>
+      </c>
+      <c r="AF2" t="s">
+        <v>168</v>
+      </c>
+      <c r="AG2" t="s">
+        <v>120</v>
+      </c>
+      <c r="AH2" t="s">
+        <v>120</v>
+      </c>
+      <c r="AI2" t="s">
+        <v>120</v>
+      </c>
+      <c r="AL2" t="s">
+        <v>169</v>
+      </c>
+      <c r="AM2" t="s">
+        <v>120</v>
+      </c>
+      <c r="AN2" t="s">
+        <v>120</v>
+      </c>
+      <c r="AO2" t="s">
+        <v>120</v>
+      </c>
+      <c r="AQ2" t="s">
+        <v>170</v>
+      </c>
+      <c r="AR2" t="s">
+        <v>120</v>
+      </c>
+      <c r="AS2" t="s">
+        <v>120</v>
+      </c>
+      <c r="AU2" t="s">
+        <v>171</v>
+      </c>
+      <c r="AV2" t="s">
+        <v>120</v>
+      </c>
+      <c r="AW2" t="s">
+        <v>120</v>
+      </c>
+      <c r="AX2" t="s">
+        <v>172</v>
+      </c>
+      <c r="AY2" t="s">
+        <v>120</v>
+      </c>
+      <c r="AZ2" t="s">
+        <v>120</v>
+      </c>
+      <c r="BA2" t="s">
+        <v>120</v>
+      </c>
+      <c r="BB2" t="s">
+        <v>120</v>
+      </c>
+      <c r="BC2" t="s">
+        <v>120</v>
+      </c>
+      <c r="BF2" t="s">
+        <v>94</v>
+      </c>
+      <c r="BG2" s="21">
+        <f t="shared" ref="BG2" si="1">DATE(1911+K2,L2,M2)</f>
+        <v>26657</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{86C9550C-6A85-4633-89A8-67CDC943236B}">
   <dimension ref="A1:CF2"/>
-  <sheetFormatPr defaultRowHeight="14.95" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.95"/>
   <cols>
     <col min="11" max="11" width="10.5" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="12.125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:84" s="9" customFormat="1" ht="24.65" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:84" s="9" customFormat="1" ht="24.65" customHeight="1">
       <c r="A1" s="7" t="s">
         <v>23</v>
       </c>
@@ -1550,7 +2044,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="2" spans="1:84" s="14" customFormat="1" ht="14.3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:84" s="14" customFormat="1" ht="14.3">
       <c r="A2" s="13">
         <v>17</v>
       </c>

</xml_diff>